<commit_message>
new requirements.txt & modify dependencies
</commit_message>
<xml_diff>
--- a/docs/Generated_paper/original_grammar_questions/test_grammar_1_['～たら〈〉(条件) '].xlsx
+++ b/docs/Generated_paper/original_grammar_questions/test_grammar_1_['～たら〈〉(条件) '].xlsx
@@ -467,17 +467,17 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 きのうはえいがをみました。それから、うちに（　　）、すぐねました。</t>
+          <t>: もんだい1 毎朝起きると、（ ）歯を磨きます。</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>1. かえると 2. かえって 3. かえれば 4. かえったら</t>
+          <t>1. すぐに 2. まだ 3. もう 4. あまり</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr"/>
@@ -491,12 +491,12 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 あしたあめがふったら、テニスのれんしゅうを（　　）。</t>
+          <t>: もんだい1 雨が（ ）傘を持って学校に行きます。</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>1. やめると 2. やめて 3. やめれば 4. やめます</t>
+          <t>1. 降るなら 2. 降れば 3. 降ると 4. 降ったら</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -515,17 +515,17 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 スーパーでりんごをかいました。それからみかんも（　　）、いつもあまいものをたべすぎてしまいます。</t>
+          <t>: もんだい1 宿題が（ ）すぐにテレビを見ます。</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>1. かうと 2. かって 3. かったら 4. かえば</t>
+          <t>1. 終わるなら 2. 終われば 3. 終わると 4. 終わったら</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr"/>
@@ -539,17 +539,17 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 でんわがきたら、すぐ（　　）。</t>
+          <t>: もんだい1 友達に会うと、（ ）「こんにちは」と言います。</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>1. きたので 2. きて 3. きまして 4. きます</t>
+          <t>1. いつも 2. じゅうぶんに 3. とても 4. あまり</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr"/>
@@ -563,17 +563,17 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 きょうはひるごはんをたべたら、ちょっと（　　）。</t>
+          <t>: もんだい1 映画が始まると、係員が（ ）静かにしてくださいとお願いします。</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>1. ねむくなりました 2. たべました 3. たべれば 4. たべたら</t>
+          <t>1. みんな 2. かならず 3. もう 4. あまり</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr"/>
@@ -587,17 +587,17 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 えきまであるいたら、ゆうびんきょくにも（　　）。</t>
+          <t>: もんだい1 財布を（ ）、学校の事務室に持っていきます。</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>1. あるくと 2. あるいて 3. あるけば 4. あるいたら</t>
+          <t>1. 見つけますと 2. 見つけれ 3. 見つけるなら 4. 見つけたら</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr"/>
@@ -611,17 +611,17 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 えきでともだちにであったら、いっしょに（　　）。</t>
+          <t>: もんだい1 お腹が（ ）昼ご飯を食べます。</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>1. あるくと 2. あるいて 3. あるきます 4. あるけば</t>
+          <t>1. 空くと 2. 空けば 3. 空くなら 4. 空いたら</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -635,12 +635,12 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 せんしゅうテストがもうありました。もしもっとべんきょう（　　）、いいてんがとれたかもしれません。</t>
+          <t>: もんだい1 本を（ ）友達に貸すつもりです。</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>1. すると 2. して 3. すれば 4. していたら</t>
+          <t>1. 買いますと 2. 買え 3. 買うなら 4. 買ったら</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
@@ -659,17 +659,17 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 きのう、ともだちがうちにくるとしらなかったので、へやが（　　）でした。もしやすくしておいたら、もっとよかったです。</t>
+          <t>: もんだい1 あなたが（ ）、メールを送りました。</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>1. きたない 2. きたくなって 3. きたなったら 4. きたなければ</t>
+          <t>1. 帰ると 2. 帰らなかったら 3. 帰れなかったら 4. 帰ったら</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr"/>
@@ -683,12 +683,12 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 せんしゅうからびょうきでした。もしやくを（　　）、きょうはげんきです。</t>
+          <t>: もんだい1 給料を（ ）、プレゼントを買います。</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>1. のむと 2. のんで 3. のめば 4. のんでいたら</t>
+          <t>1. もらうと 2. もらえ 3. もらうなら 4. もらったら</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
@@ -707,12 +707,12 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 あしたのてんきよほうであめが（　　）、ピクニックをちゅうしにします。</t>
+          <t>: もんだい2 スーパーでさいふを（ ）、先生に渡します。</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>1. ふったら 2. ふると 3. ふれば 4. ふった</t>
+          <t>1. 見つけたら 2. 見つけないと 3. 見つければ 4. 見つけたり</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 デパートでくつを（　　）、おかいけいをしてください。</t>
+          <t>: もんだい2 きのうえきでともだちに（ ）、いっしょにコーヒーをのみました。</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>1. 見つけたら 2. 見つけると 3. 見つけたとき 4. 見つけた</t>
+          <t>1. 会うと 2. 会ったら 3. 会えば 4. 会ったり</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr"/>
@@ -755,17 +755,17 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 えきについたら、ははに（　　）。</t>
+          <t>: もんだい2 でんわが（ ）、じしんのじゅうしょをかえます。</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>1. でんわします 2. でんわした 3. でんわする 4. でんわして</t>
+          <t>1. 鳴ると 2. 鳴れば 3. 鳴ったら 4. 鳴ったり</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E14" s="1" t="inlineStr"/>
@@ -779,17 +779,17 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 このくすりをのんだら、（　　）。</t>
+          <t>: もんだい2 まいあさねむりが（ ）、7時に目がさめます。</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>1. ねつがさがりました 2. ねつがさがる 3. ねつがさがって 4. ねつがさがり</t>
+          <t>1. 悪いと 2. 悪ければ 3. 悪かったら 4. 悪くても</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E15" s="1" t="inlineStr"/>
@@ -803,17 +803,17 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 スーパーでたいくつを（　　）、ともだちにでんわします。</t>
+          <t>: もんだい2 あしたせんせいに（ ）、レポートをだします。</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>1. かんじたら 2. かんじたなら 3. かんじたらすぐに 4. かんじた</t>
+          <t>1. 会うと 2. 会えば 3. 会ったら 4. 会ったり</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr"/>
@@ -827,17 +827,17 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 ともだちがいえにきたら、（　　）、いっしょにえいがをみましょう。</t>
+          <t>: もんだい2 このケーキを（ ）、みんなにほめられました。</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>1. じかんがあったら 2. じかんがあれば 3. じかんがあった 4. じかんがなくて</t>
+          <t>1. 作ると 2. 作れば 3. 作ったら 4. 作ったり</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr"/>
@@ -851,12 +851,12 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 あしたのしけんがおわったら、（　　）。</t>
+          <t>: もんだい2 えいがのよやくが（ ）、メールで知らせてください。</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>1. べんきょうします 2. べんきょうした 3. やすみます 4. べんきょうして</t>
+          <t>1. できると 2. できれば 3. できたら 4. できたり</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 おばあさんがとうきょうに（　　）、しんかんせんでむかえにいきます。</t>
+          <t>: もんだい2 あしたてんきが（ ）、びじゅつかんへ行きます。</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>1. くると 2. きたら 3. くれば 4. きた</t>
+          <t>1. 悪いと 2. 悪ければ 3. 悪かったら 4. 悪くないとき</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
@@ -899,17 +899,17 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 この(スイッチ)をおしたら、（　　）。だからさわらないでください。</t>
+          <t>: もんだい2 このメールを（ ）、とてもよろこびます。</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>1. ひがでました 2. ひがでる 3. ひがでた 4. ひがでます</t>
+          <t>1. 読むと 2. 読めば 3. 読んだら 4. 読んだり</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr"/>
@@ -923,17 +923,17 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 たなかさんがえきについたら、（　　）。やくそくのじかんは３じだから。</t>
+          <t>: もんだい2 りょこうのゆうびんを（ ）、またごれんらくください。</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>1. まちあわせをわすれた 2. まちあわせをわすれます 3. まちあわせをわすれて 4. まちあわせをわすれていた</t>
+          <t>1. 受け取ると 2. 受け取れば 3. 受け取ったら 4. 受け取ったり</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E21" s="1" t="inlineStr"/>

</xml_diff>

<commit_message>
Add voting machine (test version)
Add v4.1 based on the v3 (have not integrated v4); reconstruct the checking process of jap_question_generator.py
</commit_message>
<xml_diff>
--- a/docs/Generated_paper/original_grammar_questions/test_grammar_1_['～たら〈〉(条件) '].xlsx
+++ b/docs/Generated_paper/original_grammar_questions/test_grammar_1_['～たら〈〉(条件) '].xlsx
@@ -467,17 +467,17 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 家に帰ったら、すぐにご飯を( )。</t>
+          <t>: もんだい1 きのうは おそく ねた（   ）、 けさ おきたら もう ９じでした。</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>1. 食べたら 2. 食べるたら 3. 食べれば 4. 食べた</t>
+          <t>1. たら 2. なら 3. と 4. ば</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E2" s="1" t="inlineStr"/>
@@ -491,12 +491,12 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 駅に行く前に切符を買います。駅に着いたら( )、電車に乗ります。</t>
+          <t>: もんだい1 えきに つき（   ）、 きっさてんで コーヒーを のみます。</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>1. 切符を買ったら 2. たとき 3. れば 4. た</t>
+          <t>1. たら 2. なら 3. と 4. ば</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
@@ -515,17 +515,17 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 友達に会ったら、( )。</t>
+          <t>: もんだい1 スーパーに 行（   ）、 りんごを かって ください。</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>1. こんにちは言うたら 2. こんにちは言ったら 3. こんにちは言えば 4. こんにちは言った</t>
+          <t>1. いたら 2. いたら 3. いたら 4. いたら</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr"/>
@@ -539,17 +539,17 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 試験が終わったら、( )。</t>
+          <t>: もんだい1 あした てんきが よく（   ）、 こうえんに あそびに いきます。</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>1. 休みますたら 2. 休みますれば 3. 休みます 4. 休んだ</t>
+          <t>1. たら 2. なら 3. と 4. ば</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E5" s="1" t="inlineStr"/>
@@ -563,12 +563,12 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 映画が( )、友達とレストランに行きませんか。</t>
+          <t>: もんだい1 ともだちと えいがを み（   ）、 いえに かえりました。</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>1. 終わったら 2. 終わるたら 3. 終われば 4. 終わった</t>
+          <t>1. たら 2. たら 3. たら 4. たら</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
@@ -587,17 +587,17 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 メールを( )、返事をください。</t>
+          <t>: もんだい1 この くすりを のん（   ）、 ちょっと よく なりました。</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>1. 見たら 2. 見るたら 3. 見れば 4. 見た</t>
+          <t>1. だら 2. たら 3. たり 4. たれ</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E7" s="1" t="inlineStr"/>
@@ -611,12 +611,12 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 明日雨が( )、ピクニックをやめましょう。</t>
+          <t>: もんだい1 でんしゃの きっぷを わすれ（   ）、 あやまりました。</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>1. 降ったら 2. 降るたら 3. 降れば 4. 降った</t>
+          <t>1. たら 2. たら 3. たら 4. たら</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
@@ -635,12 +635,12 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 この薬を( )、元気になりますよ。</t>
+          <t>: もんだい1 かいものを す（   ）、 ゆうはんを つくります。</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>1. 飲んだら 2. 飲むたら 3. 飲めば元気になる 4. 飲んだ</t>
+          <t>1. したら 2. するなら 3. してと 4. したば</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
@@ -659,12 +659,12 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 道がわかりません。青い看板を( )、左に曲がってください。</t>
+          <t>: もんだい1 きょねん にほんに きた（   ）、 にほんごの べんきょうを はじめました。</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>1. 見たら 2. 見るたら 3. 見れば 4. 見た</t>
+          <t>1. たら 2. なら 3. と 4. ば</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
@@ -683,17 +683,17 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 今度の休みに空港に着いたら、母に電話を( )。</t>
+          <t>: もんだい1 たなかさんに でんわを かけ（   ）、 でかけて いました。</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>1. しますか 2. しました 3. します 4. してください</t>
+          <t>1. たら 2. たら 3. たら 4. たら</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr"/>
@@ -707,12 +707,12 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 朝、目が覚めたら、すぐに ( )。</t>
+          <t>: もんだい2 あした 天気が いい（  ）、 公園で ピクニックを します。</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>1. 起きる 2. 起きよう 3. 起きようとした 4. 起きている</t>
+          <t>1. たら 2. れば 3. なら 4. ても</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -731,17 +731,17 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 スーパーでパンを買ったら、牛乳も ( )。</t>
+          <t>: もんだい2 コンビニで ジュースを 買おうと したら、（  ）。</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>1. 買います 2. 買おう 3. 買った 4. 買っている</t>
+          <t>1. お金が なかった 2. お金が あります 3. お金が ありません 4. お金が ありますか</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E13" s="1" t="inlineStr"/>
@@ -755,12 +755,12 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 駅に着いたら、友達に ( )。</t>
+          <t>: もんだい2 宿題が 終わり（  ）、 テレビを 見ても いいですよ。</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>1. 電話する 2. 電話しよう 3. 電話した 4. 電話している</t>
+          <t>1. たら 2. れば 3. たら 4. たら</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 宿題が終わったら、テレビを ( )。</t>
+          <t>: もんだい2 駅に 着いたら、（  ）。</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>1. 見る 2. 見よう 3. 見た 4. 見ている</t>
+          <t>1. お母さんに 電話を します 2. お母さんに 電話を しました 3. お母さんに 電話を しますか 4. お母さんに 電話を しません</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
@@ -803,17 +803,17 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 雨が降ったら、ピクニックを( )。</t>
+          <t>: もんだい2 昨日、スーパーで 買い物を したら、（  ）。</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>1. やめます 2. やめよう 3. やめた 4. やめている</t>
+          <t>1. 安いリンゴが 売っていました 2. 安いリンゴが 売っています 3. 安いリンゴが 売っていますか 4. 安いリンゴが 売りません</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E16" s="1" t="inlineStr"/>
@@ -827,17 +827,17 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 銀行に行ったら、もう午後( ) 閉まっていた。</t>
+          <t>: もんだい2 電車に 乗ったら、（  ）。</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>1. 3時 2. 3時に 3. 3時で 4. 3時と</t>
+          <t>1. 窓から 景色が 見えました 2. 窓から 景色が 見えます 3. 窓から 景色が 見えません 4. 窓から 景色が 見えましょう</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E17" s="1" t="inlineStr"/>
@@ -851,17 +851,17 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 メールアドレスが ( ) 書いてあります。</t>
+          <t>: もんだい2 メールを 送ったら、（  ）。</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>1. に 2. が 3. で 4. と</t>
+          <t>1. 友だちが すぐに 返事を くれました 2. 友だちが 返事を くれます 3. 友だちが 返事を くれません 4. 友だちが 返事を くれましょう</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E18" s="1" t="inlineStr"/>
@@ -875,12 +875,12 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 昨日、駅で山田さんと会ったら、彼は ( ) いました。</t>
+          <t>: もんだい2 この 薬を 飲んだら、（  ）。</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>1. 急いで 2. 急いでて 3. 急いでいた 4. 急ぐ</t>
+          <t>1. 体が 元気になりました 2. 体が 元気になります 3. 体が 元気になりません 4. 体が 元気になりましょう</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
@@ -899,17 +899,17 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 「先週、田中さんの結婚式の話を聞いたら、思わずびっくり ( )。」</t>
+          <t>: もんだい2 先生が 教室に はいってきた（  ）、 みんなで 「おはようございます」と 言います。</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>1. しました 2. していました 3. してしまいました 4. ししていました</t>
+          <t>1. たら 2. れば 3. なら 4. ても</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="E20" s="1" t="inlineStr"/>
@@ -923,12 +923,12 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 駅前のカフェで友達を見かけたら、昨日借りた本を ( )。</t>
+          <t>: もんだい2 あなたの メールを もらった（  ）、 すぐに 返事を 書きました。</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>1. 忘れてしまった 2. 忘れている 3. 忘れよう 4. 忘れる</t>
+          <t>1. たら 2. れば 3. なら 4. ても</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">

</xml_diff>

<commit_message>
Add Excel parsing and revision pipeline v3.1
Added parse_excel_to_text to jap_excel_processor.py for extracting question data from Excel files. Introduced jap_question_generator.v3.1(qwen based).py, implementing an Excel-based revision workflow for Japanese question generation and quality assurance.
</commit_message>
<xml_diff>
--- a/docs/Generated_paper/original_grammar_questions/test_grammar_1_['～たら〈〉(条件) '].xlsx
+++ b/docs/Generated_paper/original_grammar_questions/test_grammar_1_['～たら〈〉(条件) '].xlsx
@@ -467,12 +467,12 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 きのうは おそく ねた（   ）、 けさ おきたら もう ９じでした。</t>
+          <t>: もんだい1 きょうはあめがふりました。きのうはあめがふっていなかったので、えいがをみませんでした。( ) あめがふったからです。</t>
         </is>
       </c>
       <c r="C2" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. なら 3. と 4. ば</t>
+          <t>1. あめがふったら 2. あめがふる 3. あめがふるなら 4. あめがふった</t>
         </is>
       </c>
       <c r="D2" s="1" t="inlineStr">
@@ -491,17 +491,17 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 えきに つき（   ）、 きっさてんで コーヒーを のみます。</t>
+          <t>: もんだい1 お母さんは「かんたんにできる」といいました。そう( )、お手伝いをします。</t>
         </is>
       </c>
       <c r="C3" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. なら 3. と 4. ば</t>
+          <t>1. いえ 2. いえたら 3. いえば 4. いえなかった</t>
         </is>
       </c>
       <c r="D3" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E3" s="1" t="inlineStr"/>
@@ -515,17 +515,17 @@
       </c>
       <c r="B4" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 スーパーに 行（   ）、 りんごを かって ください。</t>
+          <t>: もんだい1 たかしは がっこうを 卒業しました。 あの かおを みた( ) おなかが きもちわるくなりました。</t>
         </is>
       </c>
       <c r="C4" s="1" t="inlineStr">
         <is>
-          <t>1. いたら 2. いたら 3. いたら 4. いたら</t>
+          <t>1. あと 2. まえ 3. に 4. とき</t>
         </is>
       </c>
       <c r="D4" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>4</t>
         </is>
       </c>
       <c r="E4" s="1" t="inlineStr"/>
@@ -539,12 +539,12 @@
       </c>
       <c r="B5" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 あした てんきが よく（   ）、 こうえんに あそびに いきます。</t>
+          <t>: もんだい1 おやつをたべました。 おやつをたべ( ) えいがをみました。</t>
         </is>
       </c>
       <c r="C5" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. なら 3. と 4. ば</t>
+          <t>1. たら 2. た 3. る 4. たの</t>
         </is>
       </c>
       <c r="D5" s="1" t="inlineStr">
@@ -563,17 +563,17 @@
       </c>
       <c r="B6" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 ともだちと えいがを み（   ）、 いえに かえりました。</t>
+          <t>: もんだい1 せんせいは「がくせいが しつもんを した( ) こたえます」といいました。</t>
         </is>
       </c>
       <c r="C6" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. たら 3. たら 4. たら</t>
+          <t>1. と 2. たら 3. ば 4. なら</t>
         </is>
       </c>
       <c r="D6" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E6" s="1" t="inlineStr"/>
@@ -587,12 +587,12 @@
       </c>
       <c r="B7" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 この くすりを のん（   ）、 ちょっと よく なりました。</t>
+          <t>: もんだい1 いぬが おどりだした( ) おにいちゃんが おもちゃを あげました。</t>
         </is>
       </c>
       <c r="C7" s="1" t="inlineStr">
         <is>
-          <t>1. だら 2. たら 3. たり 4. たれ</t>
+          <t>1. と 2. たら 3. なら 4. ば</t>
         </is>
       </c>
       <c r="D7" s="1" t="inlineStr">
@@ -611,17 +611,17 @@
       </c>
       <c r="B8" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 でんしゃの きっぷを わすれ（   ）、 あやまりました。</t>
+          <t>: もんだい1 しゅくだいを おわらせた( ) えいがを みました。</t>
         </is>
       </c>
       <c r="C8" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. たら 3. たら 4. たら</t>
+          <t>1. と 2. なら 3. たら 4. ば</t>
         </is>
       </c>
       <c r="D8" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E8" s="1" t="inlineStr"/>
@@ -635,17 +635,17 @@
       </c>
       <c r="B9" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 かいものを す（   ）、 ゆうはんを つくります。</t>
+          <t>: もんだい1 おねえさんが おきがえを した( ) あさごはんを たべました。</t>
         </is>
       </c>
       <c r="C9" s="1" t="inlineStr">
         <is>
-          <t>1. したら 2. するなら 3. してと 4. したば</t>
+          <t>1. と 2. たら 3. なら 4. ば</t>
         </is>
       </c>
       <c r="D9" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E9" s="1" t="inlineStr"/>
@@ -659,17 +659,17 @@
       </c>
       <c r="B10" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 きょねん にほんに きた（   ）、 にほんごの べんきょうを はじめました。</t>
+          <t>: もんだい1 でんわが なった( ) でんわを とりました。</t>
         </is>
       </c>
       <c r="C10" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. なら 3. と 4. ば</t>
+          <t>1. と 2. なら 3. たら 4. ば</t>
         </is>
       </c>
       <c r="D10" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E10" s="1" t="inlineStr"/>
@@ -683,17 +683,17 @@
       </c>
       <c r="B11" s="1" t="inlineStr">
         <is>
-          <t>: もんだい1 たなかさんに でんわを かけ（   ）、 でかけて いました。</t>
+          <t>: もんだい1 あめがふった( ) ピクニックを キャンセルしました。</t>
         </is>
       </c>
       <c r="C11" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. たら 3. たら 4. たら</t>
+          <t>1. と 2. なら 3. たら 4. ば</t>
         </is>
       </c>
       <c r="D11" s="1" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>3</t>
         </is>
       </c>
       <c r="E11" s="1" t="inlineStr"/>
@@ -707,12 +707,12 @@
       </c>
       <c r="B12" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 あした 天気が いい（  ）、 公園で ピクニックを します。</t>
+          <t>: もんだい2 雨が降ったら、( )。</t>
         </is>
       </c>
       <c r="C12" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. れば 3. なら 4. ても</t>
+          <t>1. かえります 2. かえった 3. かえりたい 4. かえりません</t>
         </is>
       </c>
       <c r="D12" s="1" t="inlineStr">
@@ -731,12 +731,12 @@
       </c>
       <c r="B13" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 コンビニで ジュースを 買おうと したら、（  ）。</t>
+          <t>: もんだい2 友達が来たら、( )。</t>
         </is>
       </c>
       <c r="C13" s="1" t="inlineStr">
         <is>
-          <t>1. お金が なかった 2. お金が あります 3. お金が ありません 4. お金が ありますか</t>
+          <t>1. おもてなしします 2. おもてなししました 3. おもてなししたい 4. おもてなししません</t>
         </is>
       </c>
       <c r="D13" s="1" t="inlineStr">
@@ -755,12 +755,12 @@
       </c>
       <c r="B14" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 宿題が 終わり（  ）、 テレビを 見ても いいですよ。</t>
+          <t>: もんだい2 早く起きられたら、( )。</t>
         </is>
       </c>
       <c r="C14" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. れば 3. たら 4. たら</t>
+          <t>1. がんばれます 2. がんばりました 3. がんばりたい 4. がんばりません</t>
         </is>
       </c>
       <c r="D14" s="1" t="inlineStr">
@@ -779,12 +779,12 @@
       </c>
       <c r="B15" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 駅に 着いたら、（  ）。</t>
+          <t>: もんだい2 お母さんが帰ったら、( )。</t>
         </is>
       </c>
       <c r="C15" s="1" t="inlineStr">
         <is>
-          <t>1. お母さんに 電話を します 2. お母さんに 電話を しました 3. お母さんに 電話を しますか 4. お母さんに 電話を しません</t>
+          <t>1. おやつを食べます 2. おやつを食べた 3. おやつを食べたい 4. おやつを食べません</t>
         </is>
       </c>
       <c r="D15" s="1" t="inlineStr">
@@ -803,12 +803,12 @@
       </c>
       <c r="B16" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 昨日、スーパーで 買い物を したら、（  ）。</t>
+          <t>: もんだい2 テストが終わったら、( )。</t>
         </is>
       </c>
       <c r="C16" s="1" t="inlineStr">
         <is>
-          <t>1. 安いリンゴが 売っていました 2. 安いリンゴが 売っています 3. 安いリンゴが 売っていますか 4. 安いリンゴが 売りません</t>
+          <t>1. だいじょうぶです 2. だいじょうぶでした 3. だいじょうぶになりたい 4. だいじょうぶになりません</t>
         </is>
       </c>
       <c r="D16" s="1" t="inlineStr">
@@ -827,12 +827,12 @@
       </c>
       <c r="B17" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 電車に 乗ったら、（  ）。</t>
+          <t>: もんだい2 時間がないときは、( )。</t>
         </is>
       </c>
       <c r="C17" s="1" t="inlineStr">
         <is>
-          <t>1. 窓から 景色が 見えました 2. 窓から 景色が 見えます 3. 窓から 景色が 見えません 4. 窓から 景色が 見えましょう</t>
+          <t>1. あわてます 2. あわてました 3. あわてたい 4. あわてません</t>
         </is>
       </c>
       <c r="D17" s="1" t="inlineStr">
@@ -851,12 +851,12 @@
       </c>
       <c r="B18" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 メールを 送ったら、（  ）。</t>
+          <t>: もんだい2 メールが届いたら、( )。</t>
         </is>
       </c>
       <c r="C18" s="1" t="inlineStr">
         <is>
-          <t>1. 友だちが すぐに 返事を くれました 2. 友だちが 返事を くれます 3. 友だちが 返事を くれません 4. 友だちが 返事を くれましょう</t>
+          <t>1. すぐに返信します 2. すぐに返信しました 3. すぐに返信したい 4. すぐに返信しません</t>
         </is>
       </c>
       <c r="D18" s="1" t="inlineStr">
@@ -875,12 +875,12 @@
       </c>
       <c r="B19" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 この 薬を 飲んだら、（  ）。</t>
+          <t>: もんだい2 寒くなったら、( )。</t>
         </is>
       </c>
       <c r="C19" s="1" t="inlineStr">
         <is>
-          <t>1. 体が 元気になりました 2. 体が 元気になります 3. 体が 元気になりません 4. 体が 元気になりましょう</t>
+          <t>1. コートを着ます 2. コートを着ました 3. コートを着たい 4. コートを着ません</t>
         </is>
       </c>
       <c r="D19" s="1" t="inlineStr">
@@ -899,12 +899,12 @@
       </c>
       <c r="B20" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 先生が 教室に はいってきた（  ）、 みんなで 「おはようございます」と 言います。</t>
+          <t>: もんだい2 この本を読んだら、( )。</t>
         </is>
       </c>
       <c r="C20" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. れば 3. なら 4. ても</t>
+          <t>1. わかります 2. わかりました 3. わかりたい 4. わかりません</t>
         </is>
       </c>
       <c r="D20" s="1" t="inlineStr">
@@ -923,12 +923,12 @@
       </c>
       <c r="B21" s="1" t="inlineStr">
         <is>
-          <t>: もんだい2 あなたの メールを もらった（  ）、 すぐに 返事を 書きました。</t>
+          <t>: もんだい2 今日、会議が終わったら、( )。</t>
         </is>
       </c>
       <c r="C21" s="1" t="inlineStr">
         <is>
-          <t>1. たら 2. れば 3. なら 4. ても</t>
+          <t>1. みんなでご飯を食べます 2. みんなでご飯を食べました 3. みんなでご飯を食べたい 4. みんなでご飯を食べません</t>
         </is>
       </c>
       <c r="D21" s="1" t="inlineStr">

</xml_diff>